<commit_message>
feat: export/import backup, catalog always visible, modal not forced on load
</commit_message>
<xml_diff>
--- a/public/catalogo.xlsx
+++ b/public/catalogo.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yeres\OneDrive\Documentos\Webs\PREVENA PG\Skills\PreventaPG\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C885E5C4-D2DD-4FA8-864C-570EA7321080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ABF64EF3-6D66-264B-87CB-185B9607A222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E4E83839-31A0-4F46-9E9F-8E32836804A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="254">
   <si>
     <t>Categoría</t>
   </si>
@@ -563,9 +563,6 @@
     <t>16X19X80 LORO NE</t>
   </si>
   <si>
-    <t>16X19X100 LINAJE NE</t>
-  </si>
-  <si>
     <t>16X19X100 LINAJE BL</t>
   </si>
   <si>
@@ -792,6 +789,18 @@
   </si>
   <si>
     <t xml:space="preserve"> Chequera Mini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CT-6 SAN GRABIEL </t>
+  </si>
+  <si>
+    <t>16X19X100  NE LINAJE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DELY ½L TRANSPARENTE </t>
+  </si>
+  <si>
+    <t>DELY 1L TRANSPARENTE</t>
   </si>
 </sst>
 </file>
@@ -1173,14 +1182,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39340FD-E2ED-4F25-AF06-24139E7A2370}">
-  <dimension ref="A1:F238"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F241"/>
+  <sheetFormatPr defaultColWidth="10.76171875" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" customWidth="1"/>
-    <col min="2" max="2" width="32.21875" customWidth="1"/>
+    <col min="1" max="1" width="13.71875" customWidth="1"/>
+    <col min="2" max="2" width="32.1484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1200,7 +1209,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1210,11 +1219,14 @@
       <c r="C2" t="s">
         <v>44</v>
       </c>
+      <c r="D2">
+        <v>165</v>
+      </c>
       <c r="E2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1225,13 +1237,13 @@
         <v>44</v>
       </c>
       <c r="D3">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="E3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1242,13 +1254,13 @@
         <v>44</v>
       </c>
       <c r="D4">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="E4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1265,7 +1277,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1275,11 +1287,14 @@
       <c r="C6" t="s">
         <v>44</v>
       </c>
+      <c r="D6">
+        <v>160</v>
+      </c>
       <c r="E6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -1289,11 +1304,14 @@
       <c r="C7" t="s">
         <v>44</v>
       </c>
+      <c r="D7">
+        <v>160</v>
+      </c>
       <c r="E7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -1303,11 +1321,14 @@
       <c r="C8" t="s">
         <v>44</v>
       </c>
+      <c r="D8">
+        <v>160</v>
+      </c>
       <c r="E8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -1318,14 +1339,14 @@
         <v>44</v>
       </c>
       <c r="D9">
-        <v>250</v>
+        <v>160</v>
       </c>
       <c r="E9" t="s">
         <v>45</v>
       </c>
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1335,11 +1356,14 @@
       <c r="C10" t="s">
         <v>44</v>
       </c>
+      <c r="D10">
+        <v>160</v>
+      </c>
       <c r="E10" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -1349,11 +1373,14 @@
       <c r="C11" t="s">
         <v>44</v>
       </c>
+      <c r="D11">
+        <v>140</v>
+      </c>
       <c r="E11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -1363,11 +1390,14 @@
       <c r="C12" t="s">
         <v>44</v>
       </c>
+      <c r="D12">
+        <v>165</v>
+      </c>
       <c r="E12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -1377,11 +1407,14 @@
       <c r="C13" t="s">
         <v>44</v>
       </c>
+      <c r="D13">
+        <v>145</v>
+      </c>
       <c r="E13" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -1391,11 +1424,14 @@
       <c r="C14" t="s">
         <v>44</v>
       </c>
+      <c r="D14">
+        <v>145</v>
+      </c>
       <c r="E14" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -1405,11 +1441,14 @@
       <c r="C15" t="s">
         <v>44</v>
       </c>
+      <c r="D15">
+        <v>140</v>
+      </c>
       <c r="E15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -1419,11 +1458,14 @@
       <c r="C16" t="s">
         <v>44</v>
       </c>
+      <c r="D16">
+        <v>140</v>
+      </c>
       <c r="E16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -1433,11 +1475,14 @@
       <c r="C17" t="s">
         <v>44</v>
       </c>
+      <c r="D17">
+        <v>120</v>
+      </c>
       <c r="E17" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>2</v>
       </c>
@@ -1447,11 +1492,14 @@
       <c r="C18" t="s">
         <v>44</v>
       </c>
+      <c r="D18">
+        <v>120</v>
+      </c>
       <c r="E18" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>2</v>
       </c>
@@ -1461,25 +1509,31 @@
       <c r="C19" t="s">
         <v>44</v>
       </c>
+      <c r="D19">
+        <v>120</v>
+      </c>
       <c r="E19" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C20" t="s">
         <v>44</v>
       </c>
+      <c r="D20">
+        <v>120</v>
+      </c>
       <c r="E20" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>2</v>
       </c>
@@ -1493,7 +1547,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>2</v>
       </c>
@@ -1507,7 +1561,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -1521,7 +1575,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -1531,11 +1585,14 @@
       <c r="C24" t="s">
         <v>44</v>
       </c>
+      <c r="D24">
+        <v>105</v>
+      </c>
       <c r="E24" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -1550,7 +1607,7 @@
       </c>
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -1565,7 +1622,7 @@
       </c>
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>2</v>
       </c>
@@ -1580,7 +1637,7 @@
       </c>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>2</v>
       </c>
@@ -1590,12 +1647,15 @@
       <c r="C28" t="s">
         <v>44</v>
       </c>
+      <c r="D28">
+        <v>105</v>
+      </c>
       <c r="E28" t="s">
         <v>45</v>
       </c>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -1605,15 +1665,18 @@
       <c r="C29" t="s">
         <v>44</v>
       </c>
+      <c r="D29">
+        <v>120</v>
+      </c>
       <c r="E29" t="s">
         <v>45</v>
       </c>
       <c r="F29" s="1"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F30" s="1"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>62</v>
       </c>
@@ -1627,11 +1690,11 @@
         <v>130</v>
       </c>
       <c r="E31" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F31" s="1"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -1645,11 +1708,11 @@
         <v>110</v>
       </c>
       <c r="E32" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F32" s="1"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>62</v>
       </c>
@@ -1663,11 +1726,11 @@
         <v>130</v>
       </c>
       <c r="E33" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F33" s="1"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>62</v>
       </c>
@@ -1677,12 +1740,15 @@
       <c r="C34" t="s">
         <v>44</v>
       </c>
+      <c r="D34">
+        <v>110</v>
+      </c>
       <c r="E34" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F34" s="1"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>62</v>
       </c>
@@ -1692,12 +1758,15 @@
       <c r="C35" t="s">
         <v>44</v>
       </c>
+      <c r="D35">
+        <v>110</v>
+      </c>
       <c r="E35" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F35" s="1"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>62</v>
       </c>
@@ -1707,41 +1776,50 @@
       <c r="C36" t="s">
         <v>44</v>
       </c>
+      <c r="D36">
+        <v>95</v>
+      </c>
       <c r="E36" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F36" s="1"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>62</v>
       </c>
       <c r="B37" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C37" t="s">
         <v>44</v>
       </c>
+      <c r="D37">
+        <v>85</v>
+      </c>
       <c r="E37" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>62</v>
       </c>
       <c r="B38" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C38" t="s">
         <v>44</v>
       </c>
+      <c r="D38">
+        <v>85</v>
+      </c>
       <c r="E38" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F38" s="1"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>62</v>
       </c>
@@ -1752,14 +1830,14 @@
         <v>44</v>
       </c>
       <c r="D39">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E39" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F39" s="1"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>62</v>
       </c>
@@ -1770,14 +1848,14 @@
         <v>44</v>
       </c>
       <c r="D40">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="E40" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F40" s="1"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>62</v>
       </c>
@@ -1788,630 +1866,750 @@
         <v>44</v>
       </c>
       <c r="D41">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="E41" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F41" s="1"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>62</v>
       </c>
       <c r="B42" t="s">
-        <v>174</v>
+        <v>251</v>
       </c>
       <c r="C42" t="s">
         <v>44</v>
       </c>
       <c r="E42" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F42" s="1"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>62</v>
       </c>
       <c r="B43" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C43" t="s">
         <v>44</v>
       </c>
+      <c r="D43">
+        <v>105</v>
+      </c>
       <c r="E43" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F43" s="1"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>62</v>
       </c>
       <c r="B44" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C44" t="s">
         <v>44</v>
       </c>
+      <c r="D44">
+        <v>50</v>
+      </c>
       <c r="E44" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F44" s="1"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>62</v>
       </c>
       <c r="B45" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C45" t="s">
         <v>44</v>
       </c>
+      <c r="D45">
+        <v>80</v>
+      </c>
       <c r="E45" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F45" s="1"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>62</v>
       </c>
       <c r="B46" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C46" t="s">
         <v>44</v>
       </c>
+      <c r="D46">
+        <v>60</v>
+      </c>
       <c r="E46" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F46" s="1"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>62</v>
       </c>
       <c r="B47" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C47" t="s">
         <v>44</v>
       </c>
+      <c r="D47">
+        <v>85</v>
+      </c>
       <c r="E47" t="s">
+        <v>244</v>
+      </c>
+      <c r="F47" s="1"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F48" s="1"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>249</v>
+      </c>
+      <c r="B49" t="s">
+        <v>199</v>
+      </c>
+      <c r="C49" t="s">
+        <v>44</v>
+      </c>
+      <c r="D49">
+        <v>165</v>
+      </c>
+      <c r="E49" t="s">
+        <v>45</v>
+      </c>
+      <c r="F49" s="1"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>249</v>
+      </c>
+      <c r="B50" t="s">
+        <v>200</v>
+      </c>
+      <c r="C50" t="s">
+        <v>44</v>
+      </c>
+      <c r="D50">
+        <v>165</v>
+      </c>
+      <c r="E50" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>249</v>
+      </c>
+      <c r="B51" t="s">
+        <v>201</v>
+      </c>
+      <c r="C51" t="s">
+        <v>44</v>
+      </c>
+      <c r="D51">
+        <v>145</v>
+      </c>
+      <c r="E51" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>249</v>
+      </c>
+      <c r="B52" t="s">
+        <v>202</v>
+      </c>
+      <c r="C52" t="s">
+        <v>44</v>
+      </c>
+      <c r="D52">
+        <v>125</v>
+      </c>
+      <c r="E52" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>249</v>
+      </c>
+      <c r="B53" t="s">
+        <v>203</v>
+      </c>
+      <c r="C53" t="s">
+        <v>44</v>
+      </c>
+      <c r="D53">
+        <v>125</v>
+      </c>
+      <c r="E53" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>249</v>
+      </c>
+      <c r="B54" t="s">
+        <v>204</v>
+      </c>
+      <c r="C54" t="s">
+        <v>44</v>
+      </c>
+      <c r="D54">
+        <v>110</v>
+      </c>
+      <c r="E54" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>249</v>
+      </c>
+      <c r="B55" t="s">
+        <v>207</v>
+      </c>
+      <c r="C55" t="s">
+        <v>44</v>
+      </c>
+      <c r="D55">
+        <v>95</v>
+      </c>
+      <c r="E55" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>249</v>
+      </c>
+      <c r="B56" t="s">
+        <v>208</v>
+      </c>
+      <c r="C56" t="s">
+        <v>44</v>
+      </c>
+      <c r="E56" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>249</v>
+      </c>
+      <c r="B57" t="s">
+        <v>205</v>
+      </c>
+      <c r="C57" t="s">
+        <v>44</v>
+      </c>
+      <c r="D57">
+        <v>65</v>
+      </c>
+      <c r="E57" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>249</v>
+      </c>
+      <c r="B58" t="s">
+        <v>206</v>
+      </c>
+      <c r="C58" t="s">
+        <v>44</v>
+      </c>
+      <c r="D58">
+        <v>110</v>
+      </c>
+      <c r="E58" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>249</v>
+      </c>
+      <c r="B59" t="s">
+        <v>218</v>
+      </c>
+      <c r="C59" t="s">
+        <v>44</v>
+      </c>
+      <c r="D59">
+        <v>135</v>
+      </c>
+      <c r="E59" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>249</v>
+      </c>
+      <c r="B60" t="s">
+        <v>219</v>
+      </c>
+      <c r="C60" t="s">
+        <v>44</v>
+      </c>
+      <c r="E60" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>220</v>
+      </c>
+      <c r="B62" t="s">
+        <v>221</v>
+      </c>
+      <c r="C62" t="s">
+        <v>44</v>
+      </c>
+      <c r="D62">
+        <v>280</v>
+      </c>
+      <c r="E62" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>220</v>
+      </c>
+      <c r="B63" t="s">
+        <v>222</v>
+      </c>
+      <c r="C63" t="s">
+        <v>44</v>
+      </c>
+      <c r="D63">
+        <v>280</v>
+      </c>
+      <c r="E63" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>220</v>
+      </c>
+      <c r="B64" t="s">
+        <v>223</v>
+      </c>
+      <c r="C64" t="s">
+        <v>44</v>
+      </c>
+      <c r="D64">
+        <v>260</v>
+      </c>
+      <c r="E64" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>220</v>
+      </c>
+      <c r="B65" t="s">
+        <v>227</v>
+      </c>
+      <c r="C65" t="s">
+        <v>44</v>
+      </c>
+      <c r="D65">
+        <v>280</v>
+      </c>
+      <c r="E65" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>220</v>
+      </c>
+      <c r="B66" t="s">
+        <v>224</v>
+      </c>
+      <c r="C66" t="s">
+        <v>44</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>220</v>
+      </c>
+      <c r="B67" t="s">
+        <v>225</v>
+      </c>
+      <c r="C67" t="s">
+        <v>44</v>
+      </c>
+      <c r="D67">
+        <v>290</v>
+      </c>
+      <c r="E67" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>220</v>
+      </c>
+      <c r="B68" t="s">
+        <v>226</v>
+      </c>
+      <c r="C68" t="s">
+        <v>44</v>
+      </c>
+      <c r="D68">
+        <v>290</v>
+      </c>
+      <c r="E68" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>220</v>
+      </c>
+      <c r="B69" t="s">
+        <v>228</v>
+      </c>
+      <c r="C69" t="s">
+        <v>44</v>
+      </c>
+      <c r="D69">
+        <v>290</v>
+      </c>
+      <c r="E69" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>220</v>
+      </c>
+      <c r="B70" t="s">
+        <v>229</v>
+      </c>
+      <c r="C70" t="s">
+        <v>44</v>
+      </c>
+      <c r="D70">
+        <v>280</v>
+      </c>
+      <c r="E70" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>220</v>
+      </c>
+      <c r="B71" t="s">
+        <v>230</v>
+      </c>
+      <c r="C71" t="s">
+        <v>44</v>
+      </c>
+      <c r="D71">
+        <v>280</v>
+      </c>
+      <c r="E71" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>220</v>
+      </c>
+      <c r="B72" t="s">
+        <v>231</v>
+      </c>
+      <c r="C72" t="s">
+        <v>44</v>
+      </c>
+      <c r="D72">
+        <v>280</v>
+      </c>
+      <c r="E72" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>220</v>
+      </c>
+      <c r="B73" t="s">
+        <v>232</v>
+      </c>
+      <c r="C73" t="s">
+        <v>44</v>
+      </c>
+      <c r="D73">
+        <v>175</v>
+      </c>
+      <c r="E73" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>220</v>
+      </c>
+      <c r="B74" t="s">
+        <v>233</v>
+      </c>
+      <c r="C74" t="s">
+        <v>44</v>
+      </c>
+      <c r="D74">
         <v>245</v>
       </c>
-      <c r="F47" s="1"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="F48" s="1"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>250</v>
-      </c>
-      <c r="B49" t="s">
-        <v>200</v>
-      </c>
-      <c r="C49" t="s">
-        <v>44</v>
-      </c>
-      <c r="E49" t="s">
-        <v>45</v>
-      </c>
-      <c r="F49" s="1"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>250</v>
-      </c>
-      <c r="B50" t="s">
-        <v>201</v>
-      </c>
-      <c r="C50" t="s">
-        <v>44</v>
-      </c>
-      <c r="E50" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>250</v>
-      </c>
-      <c r="B51" t="s">
+      <c r="E74" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>220</v>
+      </c>
+      <c r="B75" t="s">
+        <v>234</v>
+      </c>
+      <c r="C75" t="s">
+        <v>44</v>
+      </c>
+      <c r="D75">
+        <v>245</v>
+      </c>
+      <c r="E75" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>220</v>
+      </c>
+      <c r="B76" t="s">
+        <v>235</v>
+      </c>
+      <c r="C76" t="s">
+        <v>44</v>
+      </c>
+      <c r="D76">
+        <v>245</v>
+      </c>
+      <c r="E76" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>220</v>
+      </c>
+      <c r="B77" t="s">
+        <v>239</v>
+      </c>
+      <c r="C77" t="s">
+        <v>44</v>
+      </c>
+      <c r="D77">
+        <v>245</v>
+      </c>
+      <c r="E77" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>220</v>
+      </c>
+      <c r="B78" t="s">
+        <v>236</v>
+      </c>
+      <c r="C78" t="s">
+        <v>44</v>
+      </c>
+      <c r="D78">
+        <v>245</v>
+      </c>
+      <c r="E78" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>220</v>
+      </c>
+      <c r="B79" t="s">
+        <v>237</v>
+      </c>
+      <c r="C79" t="s">
+        <v>44</v>
+      </c>
+      <c r="D79">
+        <v>245</v>
+      </c>
+      <c r="E79" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>220</v>
+      </c>
+      <c r="B80" t="s">
+        <v>238</v>
+      </c>
+      <c r="C80" t="s">
+        <v>44</v>
+      </c>
+      <c r="D80">
+        <v>245</v>
+      </c>
+      <c r="E80" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>196</v>
+      </c>
+      <c r="B82" t="s">
+        <v>195</v>
+      </c>
+      <c r="C82" t="s">
+        <v>44</v>
+      </c>
+      <c r="D82">
+        <v>180</v>
+      </c>
+      <c r="E82" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>196</v>
+      </c>
+      <c r="B83" t="s">
+        <v>194</v>
+      </c>
+      <c r="C83" t="s">
+        <v>44</v>
+      </c>
+      <c r="D83">
+        <v>227</v>
+      </c>
+      <c r="E83" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>196</v>
+      </c>
+      <c r="B84" t="s">
+        <v>193</v>
+      </c>
+      <c r="C84" t="s">
+        <v>44</v>
+      </c>
+      <c r="D84">
+        <v>190</v>
+      </c>
+      <c r="E84" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>196</v>
+      </c>
+      <c r="B85" t="s">
+        <v>192</v>
+      </c>
+      <c r="C85" t="s">
+        <v>44</v>
+      </c>
+      <c r="D85">
+        <v>259</v>
+      </c>
+      <c r="E85" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>196</v>
+      </c>
+      <c r="B86" t="s">
+        <v>191</v>
+      </c>
+      <c r="C86" t="s">
+        <v>44</v>
+      </c>
+      <c r="D86">
+        <v>181</v>
+      </c>
+      <c r="E86" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>196</v>
+      </c>
+      <c r="B87" t="s">
+        <v>190</v>
+      </c>
+      <c r="C87" t="s">
+        <v>44</v>
+      </c>
+      <c r="D87">
         <v>202</v>
       </c>
-      <c r="C51" t="s">
-        <v>44</v>
-      </c>
-      <c r="E51" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>250</v>
-      </c>
-      <c r="B52" t="s">
-        <v>203</v>
-      </c>
-      <c r="C52" t="s">
-        <v>44</v>
-      </c>
-      <c r="E52" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>250</v>
-      </c>
-      <c r="B53" t="s">
-        <v>204</v>
-      </c>
-      <c r="C53" t="s">
-        <v>44</v>
-      </c>
-      <c r="E53" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>250</v>
-      </c>
-      <c r="B54" t="s">
-        <v>205</v>
-      </c>
-      <c r="C54" t="s">
-        <v>44</v>
-      </c>
-      <c r="E54" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>250</v>
-      </c>
-      <c r="B55" t="s">
-        <v>208</v>
-      </c>
-      <c r="C55" t="s">
-        <v>44</v>
-      </c>
-      <c r="E55" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>250</v>
-      </c>
-      <c r="B56" t="s">
-        <v>209</v>
-      </c>
-      <c r="C56" t="s">
-        <v>44</v>
-      </c>
-      <c r="E56" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>250</v>
-      </c>
-      <c r="B57" t="s">
-        <v>206</v>
-      </c>
-      <c r="C57" t="s">
-        <v>44</v>
-      </c>
-      <c r="E57" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>250</v>
-      </c>
-      <c r="B58" t="s">
-        <v>207</v>
-      </c>
-      <c r="C58" t="s">
-        <v>44</v>
-      </c>
-      <c r="E58" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>250</v>
-      </c>
-      <c r="B59" t="s">
-        <v>219</v>
-      </c>
-      <c r="C59" t="s">
-        <v>44</v>
-      </c>
-      <c r="E59" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>250</v>
-      </c>
-      <c r="B60" t="s">
-        <v>220</v>
-      </c>
-      <c r="C60" t="s">
-        <v>44</v>
-      </c>
-      <c r="E60" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>221</v>
-      </c>
-      <c r="B62" t="s">
-        <v>222</v>
-      </c>
-      <c r="C62" t="s">
-        <v>44</v>
-      </c>
-      <c r="E62" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>221</v>
-      </c>
-      <c r="B63" t="s">
-        <v>223</v>
-      </c>
-      <c r="C63" t="s">
-        <v>44</v>
-      </c>
-      <c r="E63" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>221</v>
-      </c>
-      <c r="B64" t="s">
-        <v>224</v>
-      </c>
-      <c r="C64" t="s">
-        <v>44</v>
-      </c>
-      <c r="E64" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>221</v>
-      </c>
-      <c r="B65" t="s">
-        <v>228</v>
-      </c>
-      <c r="C65" t="s">
-        <v>44</v>
-      </c>
-      <c r="E65" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>221</v>
-      </c>
-      <c r="B66" t="s">
-        <v>225</v>
-      </c>
-      <c r="C66" t="s">
-        <v>44</v>
-      </c>
-      <c r="E66" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
-        <v>221</v>
-      </c>
-      <c r="B67" t="s">
-        <v>226</v>
-      </c>
-      <c r="C67" t="s">
-        <v>44</v>
-      </c>
-      <c r="E67" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>221</v>
-      </c>
-      <c r="B68" t="s">
-        <v>227</v>
-      </c>
-      <c r="C68" t="s">
-        <v>44</v>
-      </c>
-      <c r="E68" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>221</v>
-      </c>
-      <c r="B69" t="s">
-        <v>229</v>
-      </c>
-      <c r="C69" t="s">
-        <v>44</v>
-      </c>
-      <c r="E69" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>221</v>
-      </c>
-      <c r="B70" t="s">
-        <v>230</v>
-      </c>
-      <c r="C70" t="s">
-        <v>44</v>
-      </c>
-      <c r="E70" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>221</v>
-      </c>
-      <c r="B71" t="s">
-        <v>231</v>
-      </c>
-      <c r="C71" t="s">
-        <v>44</v>
-      </c>
-      <c r="E71" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>221</v>
-      </c>
-      <c r="B72" t="s">
-        <v>232</v>
-      </c>
-      <c r="C72" t="s">
-        <v>44</v>
-      </c>
-      <c r="E72" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>221</v>
-      </c>
-      <c r="B73" t="s">
-        <v>233</v>
-      </c>
-      <c r="C73" t="s">
-        <v>44</v>
-      </c>
-      <c r="E73" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
-        <v>221</v>
-      </c>
-      <c r="B74" t="s">
-        <v>234</v>
-      </c>
-      <c r="C74" t="s">
-        <v>44</v>
-      </c>
-      <c r="E74" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
-        <v>221</v>
-      </c>
-      <c r="B75" t="s">
-        <v>235</v>
-      </c>
-      <c r="C75" t="s">
-        <v>44</v>
-      </c>
-      <c r="E75" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>221</v>
-      </c>
-      <c r="B76" t="s">
-        <v>236</v>
-      </c>
-      <c r="C76" t="s">
-        <v>44</v>
-      </c>
-      <c r="E76" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>221</v>
-      </c>
-      <c r="B77" t="s">
-        <v>240</v>
-      </c>
-      <c r="C77" t="s">
-        <v>44</v>
-      </c>
-      <c r="E77" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>221</v>
-      </c>
-      <c r="B78" t="s">
-        <v>237</v>
-      </c>
-      <c r="C78" t="s">
-        <v>44</v>
-      </c>
-      <c r="E78" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>221</v>
-      </c>
-      <c r="B79" t="s">
-        <v>238</v>
-      </c>
-      <c r="C79" t="s">
-        <v>44</v>
-      </c>
-      <c r="E79" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
-        <v>221</v>
-      </c>
-      <c r="B80" t="s">
-        <v>239</v>
-      </c>
-      <c r="C80" t="s">
-        <v>44</v>
-      </c>
-      <c r="E80" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
-        <v>197</v>
-      </c>
-      <c r="B82" t="s">
-        <v>196</v>
-      </c>
-      <c r="C82" t="s">
-        <v>44</v>
-      </c>
-      <c r="E82" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>197</v>
-      </c>
-      <c r="B83" t="s">
-        <v>195</v>
-      </c>
-      <c r="C83" t="s">
-        <v>44</v>
-      </c>
-      <c r="E83" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>197</v>
-      </c>
-      <c r="B84" t="s">
-        <v>194</v>
-      </c>
-      <c r="C84" t="s">
-        <v>44</v>
-      </c>
-      <c r="E84" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>197</v>
-      </c>
-      <c r="B85" t="s">
-        <v>193</v>
-      </c>
-      <c r="C85" t="s">
-        <v>44</v>
-      </c>
-      <c r="E85" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
-        <v>197</v>
-      </c>
-      <c r="B86" t="s">
-        <v>192</v>
-      </c>
-      <c r="C86" t="s">
-        <v>44</v>
-      </c>
-      <c r="E86" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
-        <v>197</v>
-      </c>
-      <c r="B87" t="s">
-        <v>191</v>
-      </c>
-      <c r="C87" t="s">
-        <v>44</v>
-      </c>
       <c r="E87" t="s">
         <v>45</v>
       </c>
       <c r="F87" s="1"/>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F88" s="1"/>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>77</v>
       </c>
@@ -2421,12 +2619,17 @@
       <c r="C89" t="s">
         <v>44</v>
       </c>
+      <c r="D89">
+        <v>590</v>
+      </c>
       <c r="E89" t="s">
         <v>45</v>
       </c>
-      <c r="F89" s="1"/>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F89" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>77</v>
       </c>
@@ -2436,12 +2639,17 @@
       <c r="C90" t="s">
         <v>44</v>
       </c>
+      <c r="D90">
+        <v>590</v>
+      </c>
       <c r="E90" t="s">
         <v>45</v>
       </c>
-      <c r="F90" s="1"/>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F90" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>77</v>
       </c>
@@ -2451,12 +2659,17 @@
       <c r="C91" t="s">
         <v>44</v>
       </c>
+      <c r="D91">
+        <v>650</v>
+      </c>
       <c r="E91" t="s">
         <v>45</v>
       </c>
-      <c r="F91" s="1"/>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F91" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>77</v>
       </c>
@@ -2466,12 +2679,17 @@
       <c r="C92" t="s">
         <v>44</v>
       </c>
+      <c r="D92">
+        <v>560</v>
+      </c>
       <c r="E92" t="s">
         <v>45</v>
       </c>
-      <c r="F92" s="1"/>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F92" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>77</v>
       </c>
@@ -2481,12 +2699,17 @@
       <c r="C93" t="s">
         <v>44</v>
       </c>
+      <c r="D93">
+        <v>620</v>
+      </c>
       <c r="E93" t="s">
         <v>45</v>
       </c>
-      <c r="F93" s="1"/>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F93" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>77</v>
       </c>
@@ -2496,12 +2719,17 @@
       <c r="C94" t="s">
         <v>44</v>
       </c>
+      <c r="D94">
+        <v>535</v>
+      </c>
       <c r="E94" t="s">
         <v>45</v>
       </c>
-      <c r="F94" s="1"/>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F94" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>77</v>
       </c>
@@ -2511,12 +2739,17 @@
       <c r="C95" t="s">
         <v>44</v>
       </c>
+      <c r="D95">
+        <v>450</v>
+      </c>
       <c r="E95" t="s">
         <v>45</v>
       </c>
-      <c r="F95" s="1"/>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F95" s="1">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>77</v>
       </c>
@@ -2526,12 +2759,17 @@
       <c r="C96" t="s">
         <v>44</v>
       </c>
+      <c r="D96">
+        <v>450</v>
+      </c>
       <c r="E96" t="s">
         <v>45</v>
       </c>
-      <c r="F96" s="1"/>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F96" s="1">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>77</v>
       </c>
@@ -2546,7 +2784,7 @@
       </c>
       <c r="F97" s="1"/>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>77</v>
       </c>
@@ -2556,12 +2794,17 @@
       <c r="C98" t="s">
         <v>44</v>
       </c>
+      <c r="D98">
+        <v>680</v>
+      </c>
       <c r="E98" t="s">
         <v>45</v>
       </c>
-      <c r="F98" s="1"/>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F98" s="1">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>77</v>
       </c>
@@ -2576,7 +2819,7 @@
       </c>
       <c r="F99" s="1"/>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>77</v>
       </c>
@@ -2591,7 +2834,7 @@
       </c>
       <c r="F100" s="1"/>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>77</v>
       </c>
@@ -2606,7 +2849,7 @@
       </c>
       <c r="F101" s="1"/>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>77</v>
       </c>
@@ -2621,12 +2864,12 @@
       </c>
       <c r="F102" s="1"/>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>77</v>
       </c>
       <c r="B103" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C103" t="s">
         <v>44</v>
@@ -2636,7 +2879,7 @@
       </c>
       <c r="F103" s="1"/>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>77</v>
       </c>
@@ -2651,7 +2894,7 @@
       </c>
       <c r="F104" s="1"/>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>77</v>
       </c>
@@ -2664,9 +2907,11 @@
       <c r="E105" t="s">
         <v>45</v>
       </c>
-      <c r="F105" s="1"/>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F105" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>77</v>
       </c>
@@ -2679,9 +2924,11 @@
       <c r="E106" t="s">
         <v>45</v>
       </c>
-      <c r="F106" s="1"/>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F106" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>77</v>
       </c>
@@ -2692,10 +2939,10 @@
         <v>44</v>
       </c>
       <c r="E107" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>2</v>
       </c>
@@ -2709,10 +2956,10 @@
         <v>65</v>
       </c>
       <c r="E109" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>2</v>
       </c>
@@ -2726,10 +2973,10 @@
         <v>110</v>
       </c>
       <c r="E110" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>2</v>
       </c>
@@ -2740,13 +2987,13 @@
         <v>44</v>
       </c>
       <c r="D111">
-        <v>320</v>
+        <v>260</v>
       </c>
       <c r="E111" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>2</v>
       </c>
@@ -2757,13 +3004,13 @@
         <v>44</v>
       </c>
       <c r="D112">
-        <v>280</v>
+        <v>240</v>
       </c>
       <c r="E112" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>2</v>
       </c>
@@ -2774,13 +3021,13 @@
         <v>44</v>
       </c>
       <c r="D113">
-        <v>320</v>
+        <v>260</v>
       </c>
       <c r="E113" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>2</v>
       </c>
@@ -2791,13 +3038,13 @@
         <v>44</v>
       </c>
       <c r="D114">
-        <v>470</v>
+        <v>360</v>
       </c>
       <c r="E114" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>2</v>
       </c>
@@ -2808,13 +3055,13 @@
         <v>44</v>
       </c>
       <c r="D115">
-        <v>450</v>
+        <v>340</v>
       </c>
       <c r="E115" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>2</v>
       </c>
@@ -2825,13 +3072,13 @@
         <v>44</v>
       </c>
       <c r="D116">
-        <v>470</v>
+        <v>360</v>
       </c>
       <c r="E116" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>2</v>
       </c>
@@ -2841,11 +3088,14 @@
       <c r="C117" t="s">
         <v>44</v>
       </c>
+      <c r="D117">
+        <v>210</v>
+      </c>
       <c r="E117" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>2</v>
       </c>
@@ -2855,11 +3105,14 @@
       <c r="C118" t="s">
         <v>44</v>
       </c>
+      <c r="D118">
+        <v>340</v>
+      </c>
       <c r="E118" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>149</v>
       </c>
@@ -2869,11 +3122,14 @@
       <c r="C120" t="s">
         <v>45</v>
       </c>
+      <c r="D120">
+        <v>200</v>
+      </c>
       <c r="E120" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>149</v>
       </c>
@@ -2883,11 +3139,14 @@
       <c r="C121" t="s">
         <v>45</v>
       </c>
+      <c r="D121">
+        <v>200</v>
+      </c>
       <c r="E121" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>149</v>
       </c>
@@ -2897,11 +3156,14 @@
       <c r="C122" t="s">
         <v>45</v>
       </c>
+      <c r="D122">
+        <v>200</v>
+      </c>
       <c r="E122" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>149</v>
       </c>
@@ -2911,11 +3173,14 @@
       <c r="C123" t="s">
         <v>45</v>
       </c>
+      <c r="D123">
+        <v>220</v>
+      </c>
       <c r="E123" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>149</v>
       </c>
@@ -2925,11 +3190,14 @@
       <c r="C124" t="s">
         <v>45</v>
       </c>
+      <c r="D124">
+        <v>230</v>
+      </c>
       <c r="E124" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>149</v>
       </c>
@@ -2940,10 +3208,10 @@
         <v>45</v>
       </c>
       <c r="E125" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>43</v>
       </c>
@@ -2953,8 +3221,11 @@
       <c r="C127" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D127">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>43</v>
       </c>
@@ -2964,8 +3235,11 @@
       <c r="C128" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D128">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>43</v>
       </c>
@@ -2979,7 +3253,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>43</v>
       </c>
@@ -2993,7 +3267,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>43</v>
       </c>
@@ -3007,12 +3281,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>43</v>
       </c>
       <c r="B132" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C132" t="s">
         <v>45</v>
@@ -3021,12 +3295,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>43</v>
       </c>
       <c r="B133" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C133" t="s">
         <v>44</v>
@@ -3034,13 +3308,16 @@
       <c r="E133" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F133">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>43</v>
       </c>
       <c r="B134" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C134" t="s">
         <v>44</v>
@@ -3048,13 +3325,16 @@
       <c r="E134" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F134">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>43</v>
       </c>
       <c r="B135" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C135" t="s">
         <v>44</v>
@@ -3062,13 +3342,16 @@
       <c r="E135" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F135">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>43</v>
       </c>
       <c r="B136" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C136" t="s">
         <v>44</v>
@@ -3076,13 +3359,16 @@
       <c r="E136" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F136">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>43</v>
       </c>
       <c r="B137" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C137" t="s">
         <v>44</v>
@@ -3091,12 +3377,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>43</v>
       </c>
       <c r="B138" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C138" t="s">
         <v>44</v>
@@ -3105,62 +3391,71 @@
         <v>45</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>43</v>
       </c>
       <c r="B139" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C139" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>43</v>
       </c>
       <c r="B140" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C140" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>43</v>
       </c>
       <c r="B141" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C141" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D141">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>43</v>
       </c>
       <c r="B142" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C142" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D142">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>43</v>
       </c>
       <c r="B143" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C143" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D143">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>43</v>
       </c>
@@ -3171,10 +3466,10 @@
         <v>45</v>
       </c>
       <c r="D144">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>43</v>
       </c>
@@ -3185,10 +3480,10 @@
         <v>45</v>
       </c>
       <c r="D145">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>43</v>
       </c>
@@ -3199,10 +3494,10 @@
         <v>45</v>
       </c>
       <c r="D146">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>43</v>
       </c>
@@ -3213,10 +3508,10 @@
         <v>45</v>
       </c>
       <c r="D147">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>43</v>
       </c>
@@ -3227,10 +3522,10 @@
         <v>45</v>
       </c>
       <c r="D148">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>43</v>
       </c>
@@ -3241,10 +3536,10 @@
         <v>45</v>
       </c>
       <c r="D149">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>43</v>
       </c>
@@ -3255,10 +3550,10 @@
         <v>45</v>
       </c>
       <c r="D150">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>43</v>
       </c>
@@ -3269,10 +3564,10 @@
         <v>45</v>
       </c>
       <c r="D151">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>43</v>
       </c>
@@ -3286,10 +3581,10 @@
         <v>1100</v>
       </c>
       <c r="E152" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>43</v>
       </c>
@@ -3300,13 +3595,13 @@
         <v>45</v>
       </c>
       <c r="D153">
-        <v>600</v>
+        <v>650</v>
       </c>
       <c r="E153" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>43</v>
       </c>
@@ -3317,13 +3612,13 @@
         <v>45</v>
       </c>
       <c r="D154">
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="E154" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>43</v>
       </c>
@@ -3334,13 +3629,13 @@
         <v>45</v>
       </c>
       <c r="D155">
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="E155" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>43</v>
       </c>
@@ -3354,10 +3649,10 @@
         <v>320</v>
       </c>
       <c r="E156" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>43</v>
       </c>
@@ -3368,13 +3663,13 @@
         <v>45</v>
       </c>
       <c r="D157">
-        <v>320</v>
+        <v>410</v>
       </c>
       <c r="E157" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>43</v>
       </c>
@@ -3385,97 +3680,94 @@
         <v>45</v>
       </c>
       <c r="D158">
+        <v>390</v>
+      </c>
+      <c r="E158" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A159" t="s">
+        <v>43</v>
+      </c>
+      <c r="B159" t="s">
+        <v>250</v>
+      </c>
+      <c r="C159" t="s">
+        <v>45</v>
+      </c>
+      <c r="D159">
         <v>320</v>
       </c>
-      <c r="E158" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B160" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="C160" t="s">
-        <v>44</v>
-      </c>
-      <c r="E160" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="D160">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B161" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="C161" t="s">
-        <v>44</v>
-      </c>
-      <c r="E161" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A162" t="s">
-        <v>50</v>
-      </c>
-      <c r="B162" t="s">
-        <v>5</v>
-      </c>
-      <c r="C162" t="s">
-        <v>44</v>
-      </c>
-      <c r="D162">
-        <v>260</v>
-      </c>
-      <c r="E162" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="163" spans="1:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="D161">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>50</v>
       </c>
       <c r="B163" t="s">
-        <v>6</v>
+        <v>242</v>
       </c>
       <c r="C163" t="s">
         <v>44</v>
       </c>
       <c r="D163">
-        <v>260</v>
+        <v>135</v>
       </c>
       <c r="E163" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>50</v>
       </c>
       <c r="B164" t="s">
-        <v>7</v>
+        <v>243</v>
       </c>
       <c r="C164" t="s">
         <v>44</v>
       </c>
       <c r="D164">
-        <v>260</v>
+        <v>135</v>
       </c>
       <c r="E164" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>50</v>
       </c>
       <c r="B165" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C165" t="s">
         <v>44</v>
@@ -3484,15 +3776,15 @@
         <v>260</v>
       </c>
       <c r="E165" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>50</v>
       </c>
       <c r="B166" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C166" t="s">
         <v>44</v>
@@ -3501,490 +3793,580 @@
         <v>260</v>
       </c>
       <c r="E166" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>50</v>
       </c>
       <c r="B167" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C167" t="s">
         <v>44</v>
       </c>
       <c r="D167">
-        <v>320</v>
+        <v>260</v>
       </c>
       <c r="E167" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>50</v>
       </c>
       <c r="B168" t="s">
-        <v>241</v>
+        <v>8</v>
       </c>
       <c r="C168" t="s">
         <v>44</v>
       </c>
+      <c r="D168">
+        <v>260</v>
+      </c>
       <c r="E168" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>50</v>
       </c>
       <c r="B169" t="s">
-        <v>242</v>
+        <v>9</v>
       </c>
       <c r="C169" t="s">
         <v>44</v>
       </c>
+      <c r="D169">
+        <v>260</v>
+      </c>
       <c r="E169" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>50</v>
       </c>
       <c r="B170" t="s">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="C170" t="s">
         <v>44</v>
       </c>
+      <c r="D170">
+        <v>320</v>
+      </c>
       <c r="E170" t="s">
-        <v>245</v>
-      </c>
-      <c r="F170" s="1"/>
-    </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>50</v>
       </c>
       <c r="B171" t="s">
-        <v>52</v>
+        <v>240</v>
       </c>
       <c r="C171" t="s">
         <v>44</v>
       </c>
+      <c r="D171">
+        <v>125</v>
+      </c>
       <c r="E171" t="s">
-        <v>245</v>
-      </c>
-      <c r="F171" s="1"/>
-    </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>50</v>
       </c>
       <c r="B172" t="s">
-        <v>53</v>
+        <v>241</v>
       </c>
       <c r="C172" t="s">
         <v>44</v>
       </c>
+      <c r="D172">
+        <v>125</v>
+      </c>
       <c r="E172" t="s">
-        <v>245</v>
-      </c>
-      <c r="F172" s="1"/>
-    </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>50</v>
       </c>
       <c r="B173" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C173" t="s">
         <v>44</v>
       </c>
+      <c r="D173">
+        <v>210</v>
+      </c>
       <c r="E173" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F173" s="1"/>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>50</v>
       </c>
       <c r="B174" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C174" t="s">
         <v>44</v>
       </c>
+      <c r="D174">
+        <v>210</v>
+      </c>
       <c r="E174" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+      <c r="F174" s="1"/>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>50</v>
       </c>
       <c r="B175" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C175" t="s">
         <v>44</v>
       </c>
+      <c r="D175">
+        <v>210</v>
+      </c>
       <c r="E175" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+      <c r="F175" s="1"/>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>50</v>
       </c>
       <c r="B176" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C176" t="s">
         <v>44</v>
       </c>
+      <c r="D176">
+        <v>210</v>
+      </c>
       <c r="E176" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+      <c r="F176" s="1"/>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>50</v>
       </c>
       <c r="B177" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C177" t="s">
         <v>44</v>
       </c>
+      <c r="D177">
+        <v>210</v>
+      </c>
       <c r="E177" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>50</v>
       </c>
       <c r="B178" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C178" t="s">
         <v>44</v>
       </c>
+      <c r="D178">
+        <v>275</v>
+      </c>
       <c r="E178" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>50</v>
       </c>
       <c r="B179" t="s">
+        <v>57</v>
+      </c>
+      <c r="C179" t="s">
+        <v>44</v>
+      </c>
+      <c r="D179">
+        <v>190</v>
+      </c>
+      <c r="E179" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A180" t="s">
+        <v>50</v>
+      </c>
+      <c r="B180" t="s">
+        <v>58</v>
+      </c>
+      <c r="C180" t="s">
+        <v>44</v>
+      </c>
+      <c r="D180">
+        <v>190</v>
+      </c>
+      <c r="E180" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A181" t="s">
+        <v>50</v>
+      </c>
+      <c r="B181" t="s">
+        <v>59</v>
+      </c>
+      <c r="C181" t="s">
+        <v>44</v>
+      </c>
+      <c r="D181">
+        <v>190</v>
+      </c>
+      <c r="E181" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A182" t="s">
+        <v>50</v>
+      </c>
+      <c r="B182" t="s">
         <v>60</v>
       </c>
-      <c r="C179" t="s">
-        <v>44</v>
-      </c>
-      <c r="E179" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A181" t="s">
-        <v>159</v>
-      </c>
-      <c r="B181" t="s">
-        <v>160</v>
-      </c>
-      <c r="C181" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A182" t="s">
-        <v>159</v>
-      </c>
-      <c r="B182" t="s">
-        <v>162</v>
-      </c>
       <c r="C182" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A183" t="s">
-        <v>159</v>
-      </c>
-      <c r="B183" t="s">
-        <v>161</v>
-      </c>
-      <c r="C183" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+      <c r="D182">
+        <v>190</v>
+      </c>
+      <c r="E182" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>159</v>
       </c>
       <c r="B184" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C184" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D184">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A185" t="s">
+        <v>159</v>
+      </c>
+      <c r="B185" t="s">
+        <v>162</v>
+      </c>
+      <c r="C185" t="s">
+        <v>169</v>
+      </c>
+      <c r="D185">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
-        <v>78</v>
+        <v>159</v>
       </c>
       <c r="B186" t="s">
-        <v>79</v>
+        <v>161</v>
       </c>
       <c r="C186" t="s">
-        <v>44</v>
-      </c>
-      <c r="E186" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+      <c r="D186">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>78</v>
+        <v>159</v>
       </c>
       <c r="B187" t="s">
-        <v>83</v>
+        <v>163</v>
       </c>
       <c r="C187" t="s">
-        <v>44</v>
-      </c>
-      <c r="E187" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A188" t="s">
-        <v>78</v>
-      </c>
-      <c r="B188" t="s">
-        <v>80</v>
-      </c>
-      <c r="C188" t="s">
-        <v>44</v>
-      </c>
-      <c r="E188" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>78</v>
       </c>
       <c r="B189" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C189" t="s">
         <v>44</v>
       </c>
+      <c r="D189">
+        <v>75</v>
+      </c>
       <c r="E189" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>78</v>
       </c>
       <c r="B190" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C190" t="s">
         <v>44</v>
       </c>
+      <c r="D190">
+        <v>90</v>
+      </c>
       <c r="E190" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>78</v>
       </c>
       <c r="B191" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C191" t="s">
         <v>44</v>
       </c>
+      <c r="D191">
+        <v>75</v>
+      </c>
       <c r="E191" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>78</v>
       </c>
       <c r="B192" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C192" t="s">
         <v>44</v>
       </c>
+      <c r="D192">
+        <v>70</v>
+      </c>
       <c r="E192" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>78</v>
       </c>
       <c r="B193" t="s">
+        <v>82</v>
+      </c>
+      <c r="C193" t="s">
+        <v>44</v>
+      </c>
+      <c r="D193">
+        <v>70</v>
+      </c>
+      <c r="E193" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A194" t="s">
+        <v>78</v>
+      </c>
+      <c r="B194" t="s">
+        <v>84</v>
+      </c>
+      <c r="C194" t="s">
+        <v>44</v>
+      </c>
+      <c r="E194" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A195" t="s">
+        <v>78</v>
+      </c>
+      <c r="B195" t="s">
+        <v>85</v>
+      </c>
+      <c r="C195" t="s">
+        <v>44</v>
+      </c>
+      <c r="E195" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A196" t="s">
+        <v>78</v>
+      </c>
+      <c r="B196" t="s">
         <v>86</v>
       </c>
-      <c r="C193" t="s">
-        <v>44</v>
-      </c>
-      <c r="E193" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A195" t="s">
-        <v>87</v>
-      </c>
-      <c r="B195" t="s">
-        <v>88</v>
-      </c>
-      <c r="C195" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A196" t="s">
-        <v>87</v>
-      </c>
-      <c r="B196" t="s">
-        <v>89</v>
-      </c>
       <c r="C196" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A197" t="s">
-        <v>87</v>
-      </c>
-      <c r="B197" t="s">
-        <v>90</v>
-      </c>
-      <c r="C197" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+      <c r="E196" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>87</v>
       </c>
       <c r="B198" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C198" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D198">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>87</v>
       </c>
       <c r="B199" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C199" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D199">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>87</v>
       </c>
       <c r="B200" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C200" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D200">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>87</v>
       </c>
       <c r="B201" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C201" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D201">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>87</v>
       </c>
       <c r="B202" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C202" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D202">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A203" t="s">
+        <v>87</v>
+      </c>
+      <c r="B203" t="s">
+        <v>93</v>
+      </c>
+      <c r="C203" t="s">
+        <v>96</v>
+      </c>
+      <c r="D203">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B204" t="s">
-        <v>247</v>
+        <v>94</v>
       </c>
       <c r="C204" t="s">
-        <v>44</v>
-      </c>
-      <c r="E204" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+      <c r="D204">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B205" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C205" t="s">
-        <v>44</v>
-      </c>
-      <c r="E205" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A206" t="s">
-        <v>97</v>
-      </c>
-      <c r="B206" t="s">
-        <v>99</v>
-      </c>
-      <c r="C206" t="s">
-        <v>44</v>
-      </c>
-      <c r="E206" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>97</v>
       </c>
       <c r="B207" t="s">
-        <v>100</v>
+        <v>246</v>
       </c>
       <c r="C207" t="s">
         <v>44</v>
@@ -3993,12 +4375,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>97</v>
       </c>
       <c r="B208" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C208" t="s">
         <v>44</v>
@@ -4006,13 +4388,16 @@
       <c r="E208" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F208">
+        <v>21.5</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>97</v>
       </c>
       <c r="B209" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C209" t="s">
         <v>44</v>
@@ -4020,13 +4405,16 @@
       <c r="E209" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F209">
+        <v>21.5</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>97</v>
       </c>
       <c r="B210" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C210" t="s">
         <v>44</v>
@@ -4034,13 +4422,16 @@
       <c r="E210" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F210">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>97</v>
       </c>
       <c r="B211" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C211" t="s">
         <v>44</v>
@@ -4048,27 +4439,33 @@
       <c r="E211" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F211">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>97</v>
       </c>
       <c r="B212" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C212" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E212" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="F212">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>97</v>
       </c>
       <c r="B213" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C213" t="s">
         <v>44</v>
@@ -4076,263 +4473,338 @@
       <c r="E213" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F213">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>97</v>
       </c>
       <c r="B214" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C214" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E214" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="F214">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>97</v>
       </c>
       <c r="B215" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C215" t="s">
         <v>45</v>
       </c>
       <c r="E215" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>97</v>
       </c>
       <c r="B216" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C216" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E216" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="F216">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>97</v>
       </c>
       <c r="B217" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C217" t="s">
-        <v>96</v>
+        <v>45</v>
+      </c>
+      <c r="D217">
+        <v>105</v>
       </c>
       <c r="E217" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>97</v>
       </c>
       <c r="B218" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C218" t="s">
-        <v>96</v>
+        <v>45</v>
       </c>
       <c r="E218" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>97</v>
       </c>
       <c r="B219" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C219" t="s">
+        <v>45</v>
+      </c>
+      <c r="E219" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A220" t="s">
+        <v>97</v>
+      </c>
+      <c r="B220" t="s">
+        <v>117</v>
+      </c>
+      <c r="C220" t="s">
         <v>96</v>
       </c>
-      <c r="E219" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E220" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="B221" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="C221" t="s">
         <v>96</v>
       </c>
       <c r="E221" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="B222" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="C222" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A223" t="s">
-        <v>108</v>
-      </c>
-      <c r="B223" t="s">
-        <v>111</v>
-      </c>
-      <c r="C223" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E222" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>108</v>
       </c>
       <c r="B224" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C224" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D224">
+        <v>270</v>
+      </c>
+      <c r="E224" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>108</v>
       </c>
       <c r="B225" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C225" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D225">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>108</v>
       </c>
       <c r="B226" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C226" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A227" t="s">
+        <v>108</v>
+      </c>
+      <c r="B227" t="s">
+        <v>112</v>
+      </c>
+      <c r="C227" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>164</v>
+        <v>108</v>
       </c>
       <c r="B228" t="s">
-        <v>165</v>
+        <v>114</v>
       </c>
       <c r="C228" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
-        <v>164</v>
+        <v>108</v>
       </c>
       <c r="B229" t="s">
-        <v>166</v>
+        <v>113</v>
       </c>
       <c r="C229" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A230" t="s">
-        <v>164</v>
-      </c>
-      <c r="B230" t="s">
-        <v>167</v>
-      </c>
-      <c r="C230" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>164</v>
       </c>
       <c r="B231" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C231" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D231">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>164</v>
       </c>
-      <c r="B232" s="2" t="s">
+      <c r="B232" t="s">
+        <v>166</v>
+      </c>
+      <c r="C232" t="s">
+        <v>169</v>
+      </c>
+      <c r="D232">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A233" t="s">
+        <v>164</v>
+      </c>
+      <c r="B233" t="s">
+        <v>167</v>
+      </c>
+      <c r="C233" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A234" t="s">
+        <v>164</v>
+      </c>
+      <c r="B234" t="s">
+        <v>168</v>
+      </c>
+      <c r="C234" t="s">
+        <v>169</v>
+      </c>
+      <c r="D234">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A235" t="s">
+        <v>164</v>
+      </c>
+      <c r="B235" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C232" t="s">
+      <c r="C235" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B233" s="2"/>
-    </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A234" t="s">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B236" s="2"/>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A237" t="s">
+        <v>211</v>
+      </c>
+      <c r="B237" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B234" s="2" t="s">
+      <c r="C237" t="s">
+        <v>216</v>
+      </c>
+      <c r="D237">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A238" t="s">
+        <v>211</v>
+      </c>
+      <c r="B238" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="C234" t="s">
+      <c r="C238" t="s">
+        <v>216</v>
+      </c>
+      <c r="D238">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B239" s="2"/>
+    </row>
+    <row r="240" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A240" t="s">
+        <v>247</v>
+      </c>
+      <c r="B240" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C240" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A235" t="s">
-        <v>212</v>
-      </c>
-      <c r="B235" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C235" t="s">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A241" t="s">
+        <v>247</v>
+      </c>
+      <c r="B241" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C241" t="s">
         <v>217</v>
-      </c>
-    </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B236" s="2"/>
-    </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A237" t="s">
-        <v>248</v>
-      </c>
-      <c r="B237" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="C237" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A238" t="s">
-        <v>248</v>
-      </c>
-      <c r="B238" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C238" t="s">
-        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>